<commit_message>
Add Markdown Buddy and a swift software section generated from the spreadsheet
software.html now gets one section per sheet of software.xlsx, in sheet
order, instead of hard-coded sections in the template. Adding a sheet and
images/software/<sheet>-icon.png adds a section; the build fails if the
icon is missing. The CV still lists all sheets together, newest first.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TM3P1Vrynx5e2nSikcddU3
</commit_message>
<xml_diff>
--- a/data/software.xlsx
+++ b/data/software.xlsx
@@ -8,7 +8,8 @@
   <sheets>
     <sheet name="python" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="javascript" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="matlab" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="swift" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="matlab" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -1228,6 +1229,82 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:G2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>github_link</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>extra_links</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>authors</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>year</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>author_roles</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Markdown Buddy</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>MacOS Finder Quick View plugin for displaying markdown and other text-based files with syntax highlighting and high-quality rendering.</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>https://github.com/ContextLab/md-buddy</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Manning JR</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>

</xml_diff>

<commit_message>
Add CDL Slides, Knowledge Map Renderer, Thunderbird Snooze and Dream Stream
The CV's software list lowercases a description's first word so it can
follow the package name; proper nouns like Android now keep their case.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TM3P1Vrynx5e2nSikcddU3
</commit_message>
<xml_diff>
--- a/data/software.xlsx
+++ b/data/software.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -530,19 +530,19 @@
       </c>
     </row>
     <row r="2" ht="119" customHeight="1">
-      <c r="A2" s="7" t="inlineStr">
-        <is>
-          <t>Claude History Surfer</t>
-        </is>
-      </c>
-      <c r="B2" s="7" t="inlineStr">
-        <is>
-          <t>Easily navigate your Claude Code prompt history.</t>
-        </is>
-      </c>
-      <c r="C2" s="7" t="inlineStr">
-        <is>
-          <t>https://github.com/ContextLab/claude-history-surfer</t>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>CDL Slides</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Our lab's software package for creating themed slides and posters.</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>https://github.com/ContextLab/cdl-slides</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -557,17 +557,17 @@
     <row r="3" ht="34" customHeight="1">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>Claude Skill Compounder</t>
+          <t>Claude History Surfer</t>
         </is>
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>A Claude Code hook that continually asks Claude to spin off insights and discoveries into new skills.</t>
+          <t>Easily navigate your Claude Code prompt history.</t>
         </is>
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>https://github.com/ContextLab/claude-skill-compounder</t>
+          <t>https://github.com/ContextLab/claude-history-surfer</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -582,17 +582,17 @@
     <row r="4" ht="34" customHeight="1">
       <c r="A4" s="7" t="inlineStr">
         <is>
-          <t>Clustrix</t>
+          <t>Claude Skill Compounder</t>
         </is>
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>Clustrix is a Python package that enables seamless distributed computing on clusters. With a simple decorator, you can execute any Python function remotely on cluster resources while automatically handling dependency management, environment setup, and result collection.</t>
+          <t>A Claude Code hook that continually asks Claude to spin off insights and discoveries into new skills.</t>
         </is>
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>https://github.com/ContextLab/clustrix</t>
+          <t>https://github.com/ContextLab/claude-skill-compounder</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -601,28 +601,23 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="5" ht="51" customHeight="1">
-      <c r="A5" s="7" t="inlineStr">
-        <is>
-          <t>llmXive</t>
-        </is>
-      </c>
-      <c r="B5" s="7" t="inlineStr">
-        <is>
-          <t>An LLM-driven system for automating scientific discovery.</t>
-        </is>
-      </c>
-      <c r="C5" s="7" t="inlineStr">
-        <is>
-          <t>https://github.com/ContextLab/llmXive</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Demo:https://context-lab.com/llmXive</t>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Knowledge Map Renderer</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Construct Blender-based renders of knowledge maps.</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>https://github.com/ContextLab/knowledge-map-renders</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -637,260 +632,315 @@
     <row r="6" ht="34" customHeight="1">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>Chatify</t>
+          <t>Clustrix</t>
         </is>
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>Add an LLM-based "teaching assistant" to Jupyter notebooks.</t>
+          <t>Clustrix is a Python package that enables seamless distributed computing on clusters. With a simple decorator, you can execute any Python function remotely on cluster resources while automatically handling dependency management, environment setup, and result collection.</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>https://github.com/ContextLab/chatify</t>
+          <t>https://github.com/ContextLab/clustrix</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Manning JR, Manjunatha H, Kording K</t>
+          <t>Manning JR</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>2023</v>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Manjunatha H: grad</t>
-        </is>
+        <v>2025</v>
       </c>
     </row>
     <row r="7" ht="34" customHeight="1">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>Davos</t>
+          <t>llmXive</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>Manage project dependencies for notebook-based projects.</t>
+          <t>An LLM-driven system for automating scientific discovery.</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>https://github.com/ContextLab/davos</t>
+          <t>https://github.com/ContextLab/llmXive</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Demo:https://context-lab.com/llmXive</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Fitzpatrick PC, Manning JR</t>
+          <t>Manning JR</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>2022</v>
+        <v>2025</v>
       </c>
     </row>
     <row r="8" ht="17" customHeight="1">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>DataWrangler</t>
+          <t>Chatify</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>Format and clean data, with a special focus on applying natural language processing models to text data.</t>
+          <t>Add an LLM-based "teaching assistant" to Jupyter notebooks.</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>https://github.com/ContextLab/data-wrangler</t>
+          <t>https://github.com/ContextLab/chatify</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Manning JR</t>
+          <t>Manning JR, Manjunatha H, Kording K</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>2021</v>
+        <v>2023</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Manjunatha H: grad</t>
+        </is>
       </c>
     </row>
     <row r="9" ht="51" customHeight="1">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>Abstract2Paper</t>
+          <t>Davos</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>Auto-generate an entire paper from a prompt or abstract.</t>
+          <t>Manage project dependencies for notebook-based projects.</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>https://github.com/ContextLab/abstract2paper</t>
+          <t>https://github.com/ContextLab/davos</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Manning JR</t>
+          <t>Fitzpatrick PC, Manning JR</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>2021</v>
+        <v>2022</v>
       </c>
     </row>
     <row r="10" ht="170" customHeight="1">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>Timecorr Toolbox</t>
+          <t>DataWrangler</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>Estimate dynamic high-order correlations in multivariate timeseries data.</t>
+          <t>Format and clean data, with a special focus on applying natural language processing models to text data.</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>https://github.com/ContextLab/timecorr</t>
+          <t>https://github.com/ContextLab/data-wrangler</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Owen LLW, Chang TH, Manning JR</t>
+          <t>Manning JR</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>2019</v>
+        <v>2021</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>SuperEEG Toolbox</t>
+          <t>Abstract2Paper</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>Infer full-brain activity patterns from a small(ish) number of ECoG electrodes using Gaussian process regression.</t>
+          <t>Auto-generate an entire paper from a prompt or abstract.</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>https://github.com/ContextLab/supereeg</t>
+          <t>https://github.com/ContextLab/abstract2paper</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Owen LLW, Heusser AC, Manning JR</t>
+          <t>Manning JR</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>2018</v>
+        <v>2021</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>Quail</t>
+          <t>Timecorr Toolbox</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>Analyze and visualize free recall data.</t>
+          <t>Estimate dynamic high-order correlations in multivariate timeseries data.</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>https://github.com/ContextLab/quail</t>
+          <t>https://github.com/ContextLab/timecorr</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Heusser AC, Fitzpatrick PC, Field CE, Ziman K, Manning JR</t>
+          <t>Owen LLW, Chang TH, Manning JR</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>2017</v>
+        <v>2019</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>HyperTools</t>
+          <t>SuperEEG Toolbox</t>
         </is>
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>Visualize and manipulate high-dimensional data. (Way better than the MATLAB version!)</t>
+          <t>Infer full-brain activity patterns from a small(ish) number of ECoG electrodes using Gaussian process regression.</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>https://github.com/ContextLab/hypertools</t>
+          <t>https://github.com/ContextLab/supereeg</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Heusser AC, Ziman K, Owen LLW, Manning JR</t>
+          <t>Owen LLW, Heusser AC, Manning JR</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>2017</v>
+        <v>2018</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>BrainIAK Toolbox</t>
+          <t>Quail</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>Collaboration with the &lt;a href="https://pni.princeton.edu/" target="_blank"&gt;Princeton Neuroscience Institute&lt;/a&gt; and &lt;a href="http://www.intel.com/content/www/us/en/research/intel-research.html" target="_blank"&gt;Intel Labs&lt;/a&gt; to implement a bunch of useful brain analysis tools, including Hierarchical Topographic Factor Analysis.</t>
+          <t>Analyze and visualize free recall data.</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>https://github.com/IntelPNI/brainiak</t>
+          <t>https://github.com/ContextLab/quail</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Capota M, Turek J, Chen P-HC, Zhu X, Manning JR, Sundaram N, Keller B, Wang Y, Shin YS</t>
+          <t>Heusser AC, Fitzpatrick PC, Field CE, Ziman K, Manning JR</t>
         </is>
       </c>
       <c r="F14" t="n">
         <v>2017</v>
       </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>Chen P-HC: grad</t>
-        </is>
-      </c>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
+          <t>HyperTools</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Visualize and manipulate high-dimensional data. (Way better than the MATLAB version!)</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>https://github.com/ContextLab/hypertools</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Heusser AC, Ziman K, Owen LLW, Manning JR</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>2017</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>BrainIAK Toolbox</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>Collaboration with the &lt;a href="https://pni.princeton.edu/" target="_blank"&gt;Princeton Neuroscience Institute&lt;/a&gt; and &lt;a href="http://www.intel.com/content/www/us/en/research/intel-research.html" target="_blank"&gt;Intel Labs&lt;/a&gt; to implement a bunch of useful brain analysis tools, including Hierarchical Topographic Factor Analysis.</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>https://github.com/IntelPNI/brainiak</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Capota M, Turek J, Chen P-HC, Zhu X, Manning JR, Sundaram N, Keller B, Wang Y, Shin YS</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>2017</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Chen P-HC: grad</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
           <t>CDL-bibliography</t>
         </is>
       </c>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="B17" s="7" t="inlineStr">
         <is>
           <t>The bibliography management system used by the Contextual Dynamics Lab.</t>
         </is>
       </c>
-      <c r="C15" s="7" t="inlineStr">
+      <c r="C17" s="7" t="inlineStr">
         <is>
           <t>https://github.com/ContextLab/CDL-bibliography</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>Manning JR</t>
-        </is>
-      </c>
-      <c r="F15" t="n">
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Manning JR</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
         <v>2016</v>
       </c>
     </row>
@@ -905,7 +955,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -959,24 +1009,19 @@
       </c>
     </row>
     <row r="2" ht="51" customHeight="1">
-      <c r="A2" s="9" t="inlineStr">
-        <is>
-          <t>Knowledge Mapper</t>
-        </is>
-      </c>
-      <c r="B2" s="9" t="inlineStr">
-        <is>
-          <t>Map out an approximation of everything you know by answering multiple-choice quiz questions.</t>
-        </is>
-      </c>
-      <c r="C2" s="9" t="inlineStr">
-        <is>
-          <t>https://github.com/ContextLab/mapper</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Demo:https://context-lab.com/mapper/</t>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Thunderbird Snooze</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Thunderbird plugin that adds a "snooze message" feature similar to Gmail.</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>https://github.com/ContextLab/thunderbird-snooze</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -989,24 +1034,24 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="9" t="inlineStr">
-        <is>
-          <t>Scheduler</t>
-        </is>
-      </c>
-      <c r="B3" s="9" t="inlineStr">
-        <is>
-          <t>A self-hosted appointment scheduling system like YouCanBook.me or Calendly, but free, open-source, and fully under your control.</t>
-        </is>
-      </c>
-      <c r="C3" s="9" t="inlineStr">
-        <is>
-          <t>https://github.com/ContextLab/scheduler</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>https://cdl-scheduler.readthedocs.io/</t>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Dream Stream</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Android and web-based application for delivering sleep-stage triggered cues to guide lucid dreaming.</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>https://github.com/ContextLab/dream-stream</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Demo:https://context-lab.com/dream-stream/</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -1021,22 +1066,22 @@
     <row r="4">
       <c r="A4" s="9" t="inlineStr">
         <is>
-          <t>LLM Geometry Visualizer</t>
+          <t>Knowledge Mapper</t>
         </is>
       </c>
       <c r="B4" s="9" t="inlineStr">
         <is>
-          <t>Understand LLMs using geometric approaches and visualizations.</t>
+          <t>Map out an approximation of everything you know by answering multiple-choice quiz questions.</t>
         </is>
       </c>
       <c r="C4" s="9" t="inlineStr">
         <is>
-          <t>https://github.com/ContextLab/llm-geometry</t>
+          <t>https://github.com/ContextLab/mapper</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Demo:https://context-lab.com/llm-geometry</t>
+          <t>Demo:https://context-lab.com/mapper/</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -1051,22 +1096,22 @@
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
         <is>
-          <t>Fourier Control Theory</t>
+          <t>Scheduler</t>
         </is>
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>An interactive demo showing that a robot arm whose joints spin at constant rates is a Fourier series, and vice versa.</t>
+          <t>A self-hosted appointment scheduling system like YouCanBook.me or Calendly, but free, open-source, and fully under your control.</t>
         </is>
       </c>
       <c r="C5" s="9" t="inlineStr">
         <is>
-          <t>https://github.com/ContextLab/fourier-control-theory</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Demo:https://context-lab.com/fourier-control-theory</t>
+          <t>https://github.com/ContextLab/scheduler</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>https://cdl-scheduler.readthedocs.io/</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -1081,22 +1126,22 @@
     <row r="6">
       <c r="A6" s="9" t="inlineStr">
         <is>
-          <t>Sky Viewer</t>
+          <t>LLM Geometry Visualizer</t>
         </is>
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>Enter a date, location, direction, and time of day, and get back an animated visualization of the stars.</t>
+          <t>Understand LLMs using geometric approaches and visualizations.</t>
         </is>
       </c>
       <c r="C6" s="9" t="inlineStr">
         <is>
-          <t>https://github.com/ContextLab/sky-viewer</t>
+          <t>https://github.com/ContextLab/llm-geometry</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Demo:https://context-lab.com/sky-viewer</t>
+          <t>Demo:https://context-lab.com/llm-geometry</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -1111,22 +1156,22 @@
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
         <is>
-          <t>Dino Trivia</t>
+          <t>Fourier Control Theory</t>
         </is>
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>A two-player dinosaur trivia game.</t>
+          <t>An interactive demo showing that a robot arm whose joints spin at constant rates is a Fourier series, and vice versa.</t>
         </is>
       </c>
       <c r="C7" s="9" t="inlineStr">
         <is>
-          <t>https://github.com/ContextLab/dino-trivia</t>
+          <t>https://github.com/ContextLab/fourier-control-theory</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Demo:https://context-lab.com/dino-trivia</t>
+          <t>Demo:https://context-lab.com/fourier-control-theory</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -1141,17 +1186,22 @@
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
         <is>
-          <t>Claude Context Bar</t>
+          <t>Sky Viewer</t>
         </is>
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>A Claude Code mod that draws the context window as a stacked bar under the prompt.</t>
+          <t>Enter a date, location, direction, and time of day, and get back an animated visualization of the stars.</t>
         </is>
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
-          <t>https://github.com/ContextLab/claude-context-bar</t>
+          <t>https://github.com/ContextLab/sky-viewer</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Demo:https://context-lab.com/sky-viewer</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -1166,22 +1216,22 @@
     <row r="9">
       <c r="A9" s="9" t="inlineStr">
         <is>
-          <t>LLM Demos</t>
+          <t>Dino Trivia</t>
         </is>
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>A collection of interactive language model demonstrations.</t>
+          <t>A two-player dinosaur trivia game.</t>
         </is>
       </c>
       <c r="C9" s="9" t="inlineStr">
         <is>
-          <t>https://github.com/ContextLab/llm-course/tree/main/demos</t>
+          <t>https://github.com/ContextLab/dino-trivia</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Demo:https://context-lab.com/llm-course/demos/</t>
+          <t>Demo:https://context-lab.com/dino-trivia</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1190,31 +1240,86 @@
         </is>
       </c>
       <c r="G9" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
         <is>
+          <t>Claude Context Bar</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>A Claude Code mod that draws the context window as a stacked bar under the prompt.</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>https://github.com/ContextLab/claude-context-bar</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Manning JR</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>LLM Demos</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>A collection of interactive language model demonstrations.</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>https://github.com/ContextLab/llm-course/tree/main/demos</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Demo:https://context-lab.com/llm-course/demos/</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Manning JR</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
           <t>autoFR</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B12" s="9" t="inlineStr">
         <is>
           <t>A verbal free recall experiment that incorporates automatic speech-to-text processing, ready-to-run on Amazon Mechanical Turk.</t>
         </is>
       </c>
-      <c r="C10" s="9" t="inlineStr">
+      <c r="C12" s="9" t="inlineStr">
         <is>
           <t>https://github.com/ContextLab/autoFR</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="F12" t="inlineStr">
         <is>
           <t>Heusser AC, Ziman K, Fitzpatrick PC, Field CE, Manning JR</t>
         </is>
       </c>
-      <c r="G10" t="n">
+      <c r="G12" t="n">
         <v>2017</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Android Scholar in a new kotlin software section
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TM3P1Vrynx5e2nSikcddU3
</commit_message>
<xml_diff>
--- a/data/software.xlsx
+++ b/data/software.xlsx
@@ -9,7 +9,8 @@
     <sheet name="python" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="javascript" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="swift" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="matlab" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="kotlin" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="matlab" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -1410,6 +1411,82 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:G2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>github_link</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>extra_links</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>authors</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>year</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>author_roles</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Android Scholar</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Android Google Scholar application.</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>https://github.com/ContextLab/android-scholar</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Manning JR</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>

</xml_diff>